<commit_message>
feat: remap shipment contact templates
</commit_message>
<xml_diff>
--- a/data/print_templates/C__contact_label__shipment.xlsx
+++ b/data/print_templates/C__contact_label__shipment.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/EdouardGonnu/asf-wms/data/print_templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FE162B4-A7FB-354E-B9CB-0112684A6F69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50AADADE-69A0-5448-987D-36301426B3F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" xr2:uid="{D41FDF60-E254-7C4C-BFC3-DDF9FE3B5742}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17400" xr2:uid="{D41FDF60-E254-7C4C-BFC3-DDF9FE3B5742}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -39,16 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="11">
-  <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>Nom</t>
-  </si>
-  <si>
-    <t>Adresse</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="10">
   <si>
     <t>Contact</t>
   </si>
@@ -59,26 +50,119 @@
     <t>Organization</t>
   </si>
   <si>
-    <t>Contact details</t>
+    <r>
+      <t>EXPEDITEUR</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> / Shipper</t>
+    </r>
   </si>
   <si>
-    <t>Address</t>
+    <r>
+      <t xml:space="preserve">Nom / </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Name</t>
+    </r>
   </si>
   <si>
-    <t>EXPEDITEUR / SHIPPER</t>
+    <r>
+      <t xml:space="preserve">Organisation / </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Organization</t>
+    </r>
   </si>
   <si>
-    <t>DESTINATAIRE / CONSIGNEE</t>
+    <r>
+      <t xml:space="preserve">Adresse / </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Address</t>
+    </r>
   </si>
   <si>
-    <t>CORRESPONDANT / LOCAL AGENT</t>
+    <r>
+      <t>TELEPHONE</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> / Phone</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">DESTINATAIRE </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>/ Consignee</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">CORRESPONDANT </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>/ Local Agent</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -100,8 +184,30 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -110,8 +216,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4"/>
+        <fgColor theme="0" tint="-0.249977111117893"/>
         <bgColor theme="4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
@@ -121,7 +233,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -130,12 +242,12 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color theme="4" tint="0.39997558519241921"/>
+      <left style="medium">
+        <color indexed="64"/>
       </left>
       <right/>
-      <top style="thin">
-        <color theme="4" tint="0.39997558519241921"/>
+      <top style="medium">
+        <color indexed="64"/>
       </top>
       <bottom/>
       <diagonal/>
@@ -143,114 +255,69 @@
     <border>
       <left/>
       <right/>
-      <top style="thin">
-        <color theme="4" tint="0.39997558519241921"/>
+      <top style="medium">
+        <color indexed="64"/>
       </top>
       <bottom/>
       <diagonal/>
     </border>
     <border>
       <left/>
-      <right style="thin">
-        <color theme="4" tint="0.39997558519241921"/>
+      <right style="medium">
+        <color indexed="64"/>
       </right>
-      <top style="thin">
-        <color theme="4" tint="0.39997558519241921"/>
+      <top style="medium">
+        <color indexed="64"/>
       </top>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color theme="4" tint="0.39994506668294322"/>
+      <left style="medium">
+        <color indexed="64"/>
       </left>
-      <right style="thin">
-        <color theme="4" tint="0.39997558519241921"/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
       </right>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color theme="4" tint="0.39994506668294322"/>
+      <left style="medium">
+        <color indexed="64"/>
       </left>
-      <right style="thin">
-        <color theme="4" tint="0.39994506668294322"/>
-      </right>
-      <top style="thin">
-        <color theme="4" tint="0.39994506668294322"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="4" tint="0.39994506668294322"/>
-      </left>
-      <right style="thin">
-        <color theme="4" tint="0.39994506668294322"/>
-      </right>
+      <right/>
       <top/>
-      <bottom style="thin">
-        <color theme="4" tint="0.39994506668294322"/>
+      <bottom style="medium">
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left/>
-      <right style="thin">
-        <color theme="4" tint="0.39997558519241921"/>
-      </right>
+      <right/>
       <top/>
-      <bottom style="thin">
-        <color theme="4" tint="0.39997558519241921"/>
+      <bottom style="medium">
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color theme="4" tint="0.39994506668294322"/>
-      </left>
-      <right style="thin">
-        <color theme="4" tint="0.39994506668294322"/>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
       </right>
       <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color theme="4" tint="0.39997558519241921"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="4" tint="0.39994506668294322"/>
-      </left>
-      <right style="thin">
-        <color theme="4" tint="0.39997558519241921"/>
-      </right>
-      <top style="thin">
-        <color theme="4" tint="0.39997558519241921"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="4" tint="0.39994506668294322"/>
-      </left>
-      <right style="thin">
-        <color theme="4" tint="0.39997558519241921"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color theme="4" tint="0.39997558519241921"/>
+      <bottom style="medium">
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
@@ -258,41 +325,43 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -631,176 +700,201 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:D21"/>
+  <dimension ref="A2:D24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="4" width="23.1640625" customWidth="1"/>
-    <col min="5" max="5" width="2.83203125" customWidth="1"/>
+    <col min="1" max="1" width="28.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.1640625" customWidth="1"/>
+    <col min="3" max="3" width="35.83203125" customWidth="1"/>
+    <col min="4" max="4" width="23.1640625" customWidth="1"/>
+    <col min="5" max="5" width="2.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="7" t="s">
+    <row r="2" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="3"/>
+      <c r="D3" s="4"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" s="6"/>
+      <c r="D4" s="7"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="C5" s="6"/>
+      <c r="D5" s="7"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="C6" s="6"/>
+      <c r="D6" s="7"/>
+    </row>
+    <row r="7" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="10"/>
+      <c r="C7" s="10"/>
+      <c r="D7" s="11"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" s="12"/>
+    </row>
+    <row r="9" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="7"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" s="1" t="s">
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A10" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B10" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C10" s="3"/>
+      <c r="D10" s="4"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A11" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="C11" s="6"/>
+      <c r="D11" s="7"/>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A12" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="C12" s="6"/>
+      <c r="D12" s="7"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A13" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="C13" s="6"/>
+      <c r="D13" s="7"/>
+    </row>
+    <row r="14" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B14" s="10"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="11"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A15" s="12"/>
+    </row>
+    <row r="16" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A17" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="B17" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C17" s="3"/>
+      <c r="D17" s="4"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A18" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B18" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="3" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="4" t="s">
+      <c r="C18" s="6"/>
+      <c r="D18" s="7"/>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A19" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="C19" s="6"/>
+      <c r="D19" s="7"/>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A20" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" s="5" t="s">
+      <c r="B20" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="C20" s="6"/>
+      <c r="D20" s="7"/>
+    </row>
+    <row r="21" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="6" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="8"/>
-      <c r="B5" s="14"/>
-      <c r="C5" s="11"/>
-      <c r="D5" s="11"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A6" s="9"/>
-      <c r="B6" s="15"/>
-      <c r="C6" s="12"/>
-      <c r="D6" s="12"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7" s="10"/>
-      <c r="B7" s="16"/>
-      <c r="C7" s="13"/>
-      <c r="D7" s="13"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9" s="7"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A12" s="8"/>
-      <c r="B12" s="14"/>
-      <c r="C12" s="11"/>
-      <c r="D12" s="11"/>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A13" s="9"/>
-      <c r="B13" s="15"/>
-      <c r="C13" s="12"/>
-      <c r="D13" s="12"/>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14" s="10"/>
-      <c r="B14" s="16"/>
-      <c r="C14" s="13"/>
-      <c r="D14" s="13"/>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A16" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="B16" s="7"/>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A18" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="C18" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="D18" s="6" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A19" s="8"/>
-      <c r="B19" s="14"/>
-      <c r="C19" s="11"/>
-      <c r="D19" s="11"/>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A20" s="9"/>
-      <c r="B20" s="15"/>
-      <c r="C20" s="12"/>
-      <c r="D20" s="12"/>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A21" s="10"/>
-      <c r="B21" s="16"/>
-      <c r="C21" s="13"/>
-      <c r="D21" s="13"/>
-    </row>
+      <c r="B21" s="10"/>
+      <c r="C21" s="10"/>
+      <c r="D21" s="11"/>
+    </row>
+    <row r="24" spans="1:4" ht="8" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="B5:B7"/>
-    <mergeCell ref="B12:B14"/>
-    <mergeCell ref="B19:B21"/>
+  <mergeCells count="15">
+    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="B21:D21"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="B19:D19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="11" scale="86" orientation="landscape" horizontalDpi="0" verticalDpi="0"/>
+  <pageSetup paperSize="11" scale="73" orientation="landscape" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>